<commit_message>
unificada base de rasgis
</commit_message>
<xml_diff>
--- a/Galeras/Rasgos_Galeras_unificado.xlsx
+++ b/Galeras/Rasgos_Galeras_unificado.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ91"/>
+  <dimension ref="A1:AT91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -657,6 +657,21 @@
           <t>_orig_row</t>
         </is>
       </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>TreeID</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>sum</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -714,7 +729,7 @@
         <v>89.80366342301087</v>
       </c>
       <c r="P2" t="n">
-        <v>89.80366342000001</v>
+        <v>89.80366342301087</v>
       </c>
       <c r="Q2" t="n">
         <v>0.218</v>
@@ -838,7 +853,7 @@
         <v>156.0138943248532</v>
       </c>
       <c r="P3" t="n">
-        <v>156.0138943</v>
+        <v>156.0138943248532</v>
       </c>
       <c r="Q3" t="n">
         <v>0.089</v>
@@ -952,7 +967,7 @@
         <v>71.43565891472868</v>
       </c>
       <c r="P4" t="n">
-        <v>71.43565891</v>
+        <v>71.43565891472868</v>
       </c>
       <c r="Q4" t="n">
         <v>0.1511111111111111</v>
@@ -1081,7 +1096,7 @@
         <v>117.4988274706868</v>
       </c>
       <c r="P5" t="n">
-        <v>117.4988275</v>
+        <v>117.4988274706868</v>
       </c>
       <c r="Q5" t="n">
         <v>0.1766666666666666</v>
@@ -1205,7 +1220,7 @@
         <v>107.0146245059289</v>
       </c>
       <c r="P6" t="n">
-        <v>107.0146245</v>
+        <v>107.0146245059289</v>
       </c>
       <c r="Q6" t="n">
         <v>0.1755555555555555</v>
@@ -1319,7 +1334,7 @@
         <v>89.0292221084954</v>
       </c>
       <c r="P7" t="n">
-        <v>89.02922211000001</v>
+        <v>89.0292221084954</v>
       </c>
       <c r="Q7" t="n">
         <v>0.2661111111111111</v>
@@ -1443,7 +1458,7 @@
         <v>91.67092465753426</v>
       </c>
       <c r="P8" t="n">
-        <v>91.67092466</v>
+        <v>91.67092465753426</v>
       </c>
       <c r="Q8" t="n">
         <v>0.3188888888888889</v>
@@ -1567,7 +1582,7 @@
         <v>104.7709196891192</v>
       </c>
       <c r="P9" t="n">
-        <v>104.7709197</v>
+        <v>104.7709196891192</v>
       </c>
       <c r="Q9" t="n">
         <v>0.2088888888888889</v>
@@ -1696,7 +1711,7 @@
         <v>123.627095709571</v>
       </c>
       <c r="P10" t="n">
-        <v>123.6270957</v>
+        <v>123.627095709571</v>
       </c>
       <c r="Q10" t="n">
         <v>0.1477777777777778</v>
@@ -1820,7 +1835,7 @@
         <v>158.2180500658762</v>
       </c>
       <c r="P11" t="n">
-        <v>158.2180501</v>
+        <v>158.2180500658762</v>
       </c>
       <c r="Q11" t="n">
         <v>0.1343333333333333</v>
@@ -1940,7 +1955,7 @@
         <v>261.5334203655352</v>
       </c>
       <c r="P12" t="n">
-        <v>261.5334204</v>
+        <v>261.5334203655352</v>
       </c>
       <c r="R12" s="4" t="inlineStr"/>
       <c r="S12" s="4" t="inlineStr"/>
@@ -2046,7 +2061,7 @@
         <v>119.3446337308347</v>
       </c>
       <c r="P13" t="n">
-        <v>119.3446337</v>
+        <v>119.3446337308347</v>
       </c>
       <c r="Q13" t="n">
         <v>0.1223333333333333</v>
@@ -2160,7 +2175,7 @@
         <v>191.1497753369945</v>
       </c>
       <c r="P14" t="n">
-        <v>191.1497753</v>
+        <v>191.1497753369945</v>
       </c>
       <c r="Q14" t="n">
         <v>0.16</v>
@@ -2284,7 +2299,7 @@
         <v>110.1928888888889</v>
       </c>
       <c r="P15" t="n">
-        <v>110.1928889</v>
+        <v>110.1928888888889</v>
       </c>
       <c r="Q15" t="n">
         <v>0.1922222222222222</v>
@@ -2408,7 +2423,7 @@
         <v>102.8064108352145</v>
       </c>
       <c r="P16" t="n">
-        <v>102.8064108</v>
+        <v>102.8064108352145</v>
       </c>
       <c r="Q16" t="n">
         <v>0.2288888888888889</v>
@@ -2527,7 +2542,7 @@
         <v>100.3440876656473</v>
       </c>
       <c r="P17" t="n">
-        <v>100.3440877</v>
+        <v>100.3440876656473</v>
       </c>
       <c r="Q17" t="n">
         <v>0.1777777777777778</v>
@@ -2646,7 +2661,7 @@
         <v>97.92234482758622</v>
       </c>
       <c r="P18" t="n">
-        <v>97.92234483</v>
+        <v>97.92234482758622</v>
       </c>
       <c r="Q18" t="n">
         <v>0.2533333333333334</v>
@@ -2770,7 +2785,7 @@
         <v>147.6483726150393</v>
       </c>
       <c r="P19" t="n">
-        <v>147.6483726</v>
+        <v>147.6483726150393</v>
       </c>
       <c r="Q19" t="n">
         <v>0.2266666666666667</v>
@@ -2894,7 +2909,7 @@
         <v>92.22308949734369</v>
       </c>
       <c r="P20" t="n">
-        <v>92.2230895</v>
+        <v>92.22308949734369</v>
       </c>
       <c r="Q20" t="n">
         <v>0.2688888888888889</v>
@@ -3142,7 +3157,7 @@
         <v>133.1317233809001</v>
       </c>
       <c r="P22" t="n">
-        <v>133.1317234</v>
+        <v>133.1317233809001</v>
       </c>
       <c r="Q22" t="n">
         <v>0.1988888888888889</v>
@@ -3266,7 +3281,7 @@
         <v>108.3446549391069</v>
       </c>
       <c r="P23" t="n">
-        <v>108.3446549</v>
+        <v>108.3446549391069</v>
       </c>
       <c r="Q23" t="n">
         <v>0.2211111111111111</v>
@@ -3388,7 +3403,7 @@
         <v>71.33951064793837</v>
       </c>
       <c r="P24" t="n">
-        <v>71.33951064999999</v>
+        <v>71.33951064793837</v>
       </c>
       <c r="Q24" t="n">
         <v>0.2844444444444444</v>
@@ -3454,6 +3469,15 @@
       </c>
       <c r="AQ24" t="n">
         <v>22</v>
+      </c>
+      <c r="AR24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS24" t="n">
+        <v>8945</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>1574.463</v>
       </c>
     </row>
     <row r="25">
@@ -3510,7 +3534,7 @@
         <v>147.4097997892518</v>
       </c>
       <c r="P25" t="n">
-        <v>147.4097998</v>
+        <v>147.4097997892518</v>
       </c>
       <c r="Q25" t="n">
         <v>0.1011111111111111</v>
@@ -3576,6 +3600,15 @@
       </c>
       <c r="AQ25" t="n">
         <v>23</v>
+      </c>
+      <c r="AR25" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>8961</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>1328.919</v>
       </c>
     </row>
     <row r="26">
@@ -3625,8 +3658,14 @@
       <c r="M26" t="n">
         <v>30.11</v>
       </c>
+      <c r="N26" t="n">
+        <v>3083.676</v>
+      </c>
+      <c r="O26" t="n">
+        <v>102.4136831617403</v>
+      </c>
       <c r="P26" t="n">
-        <v>0</v>
+        <v>102.4136831617403</v>
       </c>
       <c r="Q26" t="n">
         <v>0.1566666666666667</v>
@@ -3692,6 +3731,15 @@
       </c>
       <c r="AQ26" t="n">
         <v>24</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>8955</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>4413.434999999999</v>
       </c>
     </row>
     <row r="27">
@@ -3748,7 +3796,7 @@
         <v>127.1500877192982</v>
       </c>
       <c r="P27" t="n">
-        <v>127.1500877</v>
+        <v>127.1500877192982</v>
       </c>
       <c r="Q27" t="n">
         <v>0.1577777777777778</v>
@@ -3807,6 +3855,15 @@
       </c>
       <c r="AQ27" t="n">
         <v>25</v>
+      </c>
+      <c r="AR27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>8957</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>1449.511</v>
       </c>
     </row>
     <row r="28">
@@ -3863,7 +3920,7 @@
         <v>158.9313006697215</v>
       </c>
       <c r="P28" t="n">
-        <v>158.9313007</v>
+        <v>158.9313006697215</v>
       </c>
       <c r="Q28" t="n">
         <v>0.07777777777777778</v>
@@ -3917,6 +3974,15 @@
       </c>
       <c r="AQ28" t="n">
         <v>26</v>
+      </c>
+      <c r="AR28" t="n">
+        <v>4</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>8962</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>4548.025</v>
       </c>
     </row>
     <row r="29">
@@ -3973,7 +4039,7 @@
         <v>163.0783269961977</v>
       </c>
       <c r="P29" t="n">
-        <v>163.078327</v>
+        <v>163.0783269961977</v>
       </c>
       <c r="Q29" t="n">
         <v>0.1522222222222222</v>
@@ -4039,6 +4105,15 @@
       </c>
       <c r="AQ29" t="n">
         <v>27</v>
+      </c>
+      <c r="AR29" t="n">
+        <v>7</v>
+      </c>
+      <c r="AS29" t="n">
+        <v>8968</v>
+      </c>
+      <c r="AT29" t="n">
+        <v>428.896</v>
       </c>
     </row>
     <row r="30">
@@ -4082,9 +4157,14 @@
       <c r="M30" s="4" t="n">
         <v>31.25</v>
       </c>
-      <c r="N30" s="4" t="inlineStr"/>
+      <c r="N30" t="n">
+        <v>4099.39</v>
+      </c>
+      <c r="O30" t="n">
+        <v>131.18048</v>
+      </c>
       <c r="P30" t="n">
-        <v>0</v>
+        <v>131.18048</v>
       </c>
       <c r="Q30" t="n">
         <v>0.1611111111111111</v>
@@ -4154,6 +4234,15 @@
       <c r="AQ30" t="n">
         <v>28</v>
       </c>
+      <c r="AR30" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS30" t="n">
+        <v>8965</v>
+      </c>
+      <c r="AT30" t="n">
+        <v>4099.39</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -4203,7 +4292,7 @@
         <v>151.6336528221512</v>
       </c>
       <c r="P31" t="n">
-        <v>151.6336528</v>
+        <v>151.6336528221512</v>
       </c>
       <c r="Q31" t="n">
         <v>0.1344444444444444</v>
@@ -4273,6 +4362,15 @@
       <c r="AQ31" t="n">
         <v>29</v>
       </c>
+      <c r="AR31" t="n">
+        <v>6</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>8966</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>1423.84</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4328,7 +4426,7 @@
         <v>209.8016470588235</v>
       </c>
       <c r="P32" t="n">
-        <v>209.8016471</v>
+        <v>209.8016470588235</v>
       </c>
       <c r="Q32" t="n">
         <v>0.1288888888888889</v>
@@ -4394,6 +4492,15 @@
       </c>
       <c r="AQ32" t="n">
         <v>30</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>15</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>8986</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>1783.314</v>
       </c>
     </row>
     <row r="33">
@@ -4445,7 +4552,7 @@
         <v>74.72674113009198</v>
       </c>
       <c r="P33" t="n">
-        <v>74.72674112999999</v>
+        <v>74.72674113009198</v>
       </c>
       <c r="Q33" t="n">
         <v>0.2022222222222222</v>
@@ -4511,6 +4618,15 @@
       </c>
       <c r="AQ33" t="n">
         <v>31</v>
+      </c>
+      <c r="AR33" t="n">
+        <v>16</v>
+      </c>
+      <c r="AS33" t="n">
+        <v>8989</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>2274.682</v>
       </c>
     </row>
     <row r="34">
@@ -4567,7 +4683,7 @@
         <v>62.21783305227656</v>
       </c>
       <c r="P34" t="n">
-        <v>62.21783305</v>
+        <v>62.21783305227656</v>
       </c>
       <c r="Q34" t="n">
         <v>0.2188888888888889</v>
@@ -4633,6 +4749,15 @@
       </c>
       <c r="AQ34" t="n">
         <v>32</v>
+      </c>
+      <c r="AR34" t="n">
+        <v>13</v>
+      </c>
+      <c r="AS34" t="n">
+        <v>8983</v>
+      </c>
+      <c r="AT34" t="n">
+        <v>1475.807</v>
       </c>
     </row>
     <row r="35">
@@ -4689,7 +4814,7 @@
         <v>105.080442804428</v>
       </c>
       <c r="P35" t="n">
-        <v>105.0804428</v>
+        <v>105.080442804428</v>
       </c>
       <c r="Q35" t="n">
         <v>0.1466666666666667</v>
@@ -4755,6 +4880,15 @@
       </c>
       <c r="AQ35" t="n">
         <v>33</v>
+      </c>
+      <c r="AR35" t="n">
+        <v>12</v>
+      </c>
+      <c r="AS35" t="n">
+        <v>8982</v>
+      </c>
+      <c r="AT35" t="n">
+        <v>3417.216</v>
       </c>
     </row>
     <row r="36">
@@ -4811,7 +4945,7 @@
         <v>174.3038461538461</v>
       </c>
       <c r="P36" t="n">
-        <v>174.3038462</v>
+        <v>174.3038461538461</v>
       </c>
       <c r="Q36" t="n">
         <v>0.1433333333333333</v>
@@ -4877,6 +5011,15 @@
       </c>
       <c r="AQ36" t="n">
         <v>34</v>
+      </c>
+      <c r="AR36" t="n">
+        <v>10</v>
+      </c>
+      <c r="AS36" t="n">
+        <v>8976</v>
+      </c>
+      <c r="AT36" t="n">
+        <v>317.233</v>
       </c>
     </row>
     <row r="37">
@@ -4933,7 +5076,7 @@
         <v>84.77002491990032</v>
       </c>
       <c r="P37" t="n">
-        <v>84.77002492</v>
+        <v>84.77002491990032</v>
       </c>
       <c r="Q37" t="n">
         <v>0.1788888888888889</v>
@@ -4999,6 +5142,15 @@
       </c>
       <c r="AQ37" t="n">
         <v>35</v>
+      </c>
+      <c r="AR37" t="n">
+        <v>9</v>
+      </c>
+      <c r="AS37" t="n">
+        <v>8975</v>
+      </c>
+      <c r="AT37" t="n">
+        <v>2381.19</v>
       </c>
     </row>
     <row r="38">
@@ -5055,7 +5207,7 @@
         <v>117.4496603260869</v>
       </c>
       <c r="P38" t="n">
-        <v>117.4496603</v>
+        <v>117.4496603260869</v>
       </c>
       <c r="Q38" t="n">
         <v>0.1622222222222222</v>
@@ -5121,6 +5273,15 @@
       </c>
       <c r="AQ38" t="n">
         <v>36</v>
+      </c>
+      <c r="AR38" t="n">
+        <v>8</v>
+      </c>
+      <c r="AS38" t="n">
+        <v>8974</v>
+      </c>
+      <c r="AT38" t="n">
+        <v>1728.859</v>
       </c>
     </row>
     <row r="39">
@@ -5177,7 +5338,7 @@
         <v>121.370652173913</v>
       </c>
       <c r="P39" t="n">
-        <v>121.3706522</v>
+        <v>121.370652173913</v>
       </c>
       <c r="Q39" t="n">
         <v>0.1277777777777778</v>
@@ -5243,6 +5404,15 @@
       </c>
       <c r="AQ39" t="n">
         <v>37</v>
+      </c>
+      <c r="AR39" t="n">
+        <v>11</v>
+      </c>
+      <c r="AS39" t="n">
+        <v>8980</v>
+      </c>
+      <c r="AT39" t="n">
+        <v>1116.61</v>
       </c>
     </row>
     <row r="40">
@@ -5286,7 +5456,7 @@
         <v>191.9872602739726</v>
       </c>
       <c r="P40" t="n">
-        <v>191.9872603</v>
+        <v>191.9872602739726</v>
       </c>
       <c r="Q40" t="n">
         <v>0.1033333333333333</v>
@@ -5325,6 +5495,15 @@
       </c>
       <c r="AQ40" t="n">
         <v>38</v>
+      </c>
+      <c r="AR40" t="n">
+        <v>14</v>
+      </c>
+      <c r="AS40" t="n">
+        <v>8985</v>
+      </c>
+      <c r="AT40" t="n">
+        <v>1401.507</v>
       </c>
     </row>
     <row r="41">
@@ -5378,7 +5557,7 @@
         <v>67.86092715231788</v>
       </c>
       <c r="P41" t="n">
-        <v>67.86092714999999</v>
+        <v>67.86092715231788</v>
       </c>
       <c r="Q41" t="n">
         <v>0.2438888888888889</v>
@@ -5498,8 +5677,14 @@
       <c r="M42" t="n">
         <v>6.56</v>
       </c>
+      <c r="N42" t="n">
+        <v>864.848</v>
+      </c>
+      <c r="O42" t="n">
+        <v>131.8365853658537</v>
+      </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>131.8365853658537</v>
       </c>
       <c r="Q42" t="n">
         <v>0.1755555555555556</v>
@@ -5565,6 +5750,15 @@
       </c>
       <c r="AQ42" t="n">
         <v>40</v>
+      </c>
+      <c r="AR42" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS42" t="n">
+        <v>8738</v>
+      </c>
+      <c r="AT42" t="n">
+        <v>864.848</v>
       </c>
     </row>
     <row r="43">
@@ -5614,8 +5808,14 @@
       <c r="M43" t="n">
         <v>45.1</v>
       </c>
+      <c r="N43" t="n">
+        <v>4311.9653472</v>
+      </c>
+      <c r="O43" t="n">
+        <v>95.60898774279379</v>
+      </c>
       <c r="P43" t="n">
-        <v>0</v>
+        <v>95.60898774279379</v>
       </c>
       <c r="Q43" t="n">
         <v>0.2455555555555556</v>
@@ -5686,6 +5886,15 @@
       </c>
       <c r="AQ43" t="n">
         <v>41</v>
+      </c>
+      <c r="AR43" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS43" t="n">
+        <v>8735</v>
+      </c>
+      <c r="AT43" t="n">
+        <v>4311.9653472</v>
       </c>
     </row>
     <row r="44">
@@ -5742,7 +5951,7 @@
         <v>139.4317757009346</v>
       </c>
       <c r="P44" t="n">
-        <v>139.4317757</v>
+        <v>139.4317757009346</v>
       </c>
       <c r="Q44" t="n">
         <v>0.08555555555555555</v>
@@ -5813,6 +6022,15 @@
       </c>
       <c r="AQ44" t="n">
         <v>42</v>
+      </c>
+      <c r="AR44" t="n">
+        <v>20</v>
+      </c>
+      <c r="AS44" t="n">
+        <v>8721</v>
+      </c>
+      <c r="AT44" t="n">
+        <v>305.717</v>
       </c>
     </row>
     <row r="45">
@@ -5869,7 +6087,7 @@
         <v>117.7141830065359</v>
       </c>
       <c r="P45" t="n">
-        <v>117.714183</v>
+        <v>117.7141830065359</v>
       </c>
       <c r="Q45" t="n">
         <v>0.2077777777777778</v>
@@ -5998,7 +6216,7 @@
         <v>93.23147502903601</v>
       </c>
       <c r="P46" t="n">
-        <v>93.23147503</v>
+        <v>93.23147502903601</v>
       </c>
       <c r="Q46" t="n">
         <v>0.2886666666666666</v>
@@ -6069,6 +6287,15 @@
       </c>
       <c r="AQ46" t="n">
         <v>44</v>
+      </c>
+      <c r="AR46" t="n">
+        <v>18</v>
+      </c>
+      <c r="AS46" t="n">
+        <v>8716</v>
+      </c>
+      <c r="AT46" t="n">
+        <v>833.1849999999999</v>
       </c>
     </row>
     <row r="47">
@@ -6125,7 +6352,7 @@
         <v>65.31316337148803</v>
       </c>
       <c r="P47" t="n">
-        <v>65.31316337</v>
+        <v>65.31316337148803</v>
       </c>
       <c r="Q47" t="n">
         <v>0.21</v>
@@ -6169,6 +6396,15 @@
       </c>
       <c r="AQ47" t="n">
         <v>45</v>
+      </c>
+      <c r="AR47" t="n">
+        <v>19</v>
+      </c>
+      <c r="AS47" t="n">
+        <v>8718</v>
+      </c>
+      <c r="AT47" t="n">
+        <v>1331.401</v>
       </c>
     </row>
     <row r="48">
@@ -6218,8 +6454,14 @@
       <c r="M48" t="n">
         <v>17.16</v>
       </c>
+      <c r="N48" t="n">
+        <v>1834.82520848</v>
+      </c>
+      <c r="O48" t="n">
+        <v>106.9245459487179</v>
+      </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>106.9245459487179</v>
       </c>
       <c r="Q48" t="n">
         <v>0.2396666666666667</v>
@@ -6288,6 +6530,15 @@
       </c>
       <c r="AQ48" t="n">
         <v>46</v>
+      </c>
+      <c r="AR48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS48" t="n">
+        <v>8711</v>
+      </c>
+      <c r="AT48" t="n">
+        <v>1834.82520848</v>
       </c>
     </row>
     <row r="49">
@@ -6344,7 +6595,7 @@
         <v>97.07211474316212</v>
       </c>
       <c r="P49" t="n">
-        <v>97.07211474</v>
+        <v>97.07211474316212</v>
       </c>
       <c r="Q49" t="n">
         <v>0.2344444444444444</v>
@@ -6417,6 +6668,15 @@
       </c>
       <c r="AQ49" t="n">
         <v>47</v>
+      </c>
+      <c r="AR49" t="n">
+        <v>17</v>
+      </c>
+      <c r="AS49" t="n">
+        <v>8708</v>
+      </c>
+      <c r="AT49" t="n">
+        <v>1455.111</v>
       </c>
     </row>
     <row r="50">
@@ -6468,7 +6728,7 @@
         <v>75.99312267657993</v>
       </c>
       <c r="P50" t="n">
-        <v>75.99312268</v>
+        <v>75.99312267657993</v>
       </c>
       <c r="Q50" t="n">
         <v>0.3732222222222222</v>
@@ -6584,7 +6844,7 @@
         <v>108.3975364963504</v>
       </c>
       <c r="P51" t="n">
-        <v>108.3975365</v>
+        <v>108.3975364963504</v>
       </c>
       <c r="Q51" t="n">
         <v>0.1847777777777778</v>
@@ -6696,8 +6956,14 @@
       <c r="M52" t="n">
         <v>8.970000000000001</v>
       </c>
+      <c r="N52" t="n">
+        <v>825.0649999999999</v>
+      </c>
+      <c r="O52" t="n">
+        <v>91.98049052396877</v>
+      </c>
       <c r="P52" t="n">
-        <v>0</v>
+        <v>91.98049052396877</v>
       </c>
       <c r="Q52" t="n">
         <v>0.1455555555555555</v>
@@ -6736,6 +7002,15 @@
       </c>
       <c r="AQ52" t="n">
         <v>50</v>
+      </c>
+      <c r="AR52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS52" t="n">
+        <v>8715</v>
+      </c>
+      <c r="AT52" t="n">
+        <v>825.0649999999999</v>
       </c>
     </row>
     <row r="53">
@@ -6785,8 +7060,14 @@
       <c r="M53" t="n">
         <v>24.37</v>
       </c>
+      <c r="N53" t="n">
+        <v>2724.862</v>
+      </c>
+      <c r="O53" t="n">
+        <v>111.8121460812474</v>
+      </c>
       <c r="P53" t="n">
-        <v>0</v>
+        <v>111.8121460812474</v>
       </c>
       <c r="Q53" t="n">
         <v>0.1213333333333333</v>
@@ -6852,6 +7133,15 @@
       </c>
       <c r="AQ53" t="n">
         <v>51</v>
+      </c>
+      <c r="AR53" t="n">
+        <v>34</v>
+      </c>
+      <c r="AS53" t="n">
+        <v>8786</v>
+      </c>
+      <c r="AT53" t="n">
+        <v>2724.862</v>
       </c>
     </row>
     <row r="54">
@@ -6901,8 +7191,14 @@
       <c r="M54" t="n">
         <v>10.56</v>
       </c>
+      <c r="N54" t="n">
+        <v>1277.754</v>
+      </c>
+      <c r="O54" t="n">
+        <v>120.9994318181818</v>
+      </c>
       <c r="P54" t="n">
-        <v>0</v>
+        <v>120.9994318181818</v>
       </c>
       <c r="Q54" t="n">
         <v>0.1786666666666666</v>
@@ -6968,6 +7264,15 @@
       </c>
       <c r="AQ54" t="n">
         <v>52</v>
+      </c>
+      <c r="AR54" t="n">
+        <v>36</v>
+      </c>
+      <c r="AS54" t="n">
+        <v>8796</v>
+      </c>
+      <c r="AT54" t="n">
+        <v>1277.754</v>
       </c>
     </row>
     <row r="55">
@@ -7017,8 +7322,14 @@
       <c r="M55" t="n">
         <v>3.05</v>
       </c>
+      <c r="N55" t="n">
+        <v>320.448</v>
+      </c>
+      <c r="O55" t="n">
+        <v>105.0649180327869</v>
+      </c>
       <c r="P55" t="n">
-        <v>0</v>
+        <v>105.0649180327869</v>
       </c>
       <c r="Q55" t="n">
         <v>0.1254444444444444</v>
@@ -7084,6 +7395,15 @@
       </c>
       <c r="AQ55" t="n">
         <v>53</v>
+      </c>
+      <c r="AR55" t="n">
+        <v>37</v>
+      </c>
+      <c r="AS55" t="n">
+        <v>8800</v>
+      </c>
+      <c r="AT55" t="n">
+        <v>320.448</v>
       </c>
     </row>
     <row r="56">
@@ -7133,8 +7453,14 @@
       <c r="M56" t="n">
         <v>11.83</v>
       </c>
+      <c r="N56" t="n">
+        <v>1037.63</v>
+      </c>
+      <c r="O56" t="n">
+        <v>87.71174978867288</v>
+      </c>
       <c r="P56" t="n">
-        <v>0</v>
+        <v>87.71174978867288</v>
       </c>
       <c r="Q56" t="n">
         <v>0.1642222222222222</v>
@@ -7200,6 +7526,15 @@
       </c>
       <c r="AQ56" t="n">
         <v>54</v>
+      </c>
+      <c r="AR56" t="n">
+        <v>32</v>
+      </c>
+      <c r="AS56" t="n">
+        <v>8778</v>
+      </c>
+      <c r="AT56" t="n">
+        <v>1037.63</v>
       </c>
     </row>
     <row r="57">
@@ -7249,8 +7584,14 @@
       <c r="M57" t="n">
         <v>11.4</v>
       </c>
+      <c r="N57" t="n">
+        <v>1440.586</v>
+      </c>
+      <c r="O57" t="n">
+        <v>126.3671929824561</v>
+      </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>126.3671929824561</v>
       </c>
       <c r="Q57" t="n">
         <v>0.2394444444444445</v>
@@ -7316,6 +7657,15 @@
       </c>
       <c r="AQ57" t="n">
         <v>55</v>
+      </c>
+      <c r="AR57" t="n">
+        <v>33</v>
+      </c>
+      <c r="AS57" t="n">
+        <v>8780</v>
+      </c>
+      <c r="AT57" t="n">
+        <v>1440.586</v>
       </c>
     </row>
     <row r="58">
@@ -7365,8 +7715,14 @@
       <c r="M58" t="n">
         <v>7.31</v>
       </c>
+      <c r="N58" t="n">
+        <v>459.263</v>
+      </c>
+      <c r="O58" t="n">
+        <v>62.82667578659371</v>
+      </c>
       <c r="P58" t="n">
-        <v>0</v>
+        <v>62.82667578659371</v>
       </c>
       <c r="Q58" t="n">
         <v>0.2881111111111111</v>
@@ -7432,6 +7788,15 @@
       </c>
       <c r="AQ58" t="n">
         <v>56</v>
+      </c>
+      <c r="AR58" t="n">
+        <v>30</v>
+      </c>
+      <c r="AS58" t="n">
+        <v>8615</v>
+      </c>
+      <c r="AT58" t="n">
+        <v>459.263</v>
       </c>
     </row>
     <row r="59">
@@ -7481,8 +7846,14 @@
       <c r="M59" t="n">
         <v>15.49</v>
       </c>
+      <c r="N59" t="n">
+        <v>1068.994</v>
+      </c>
+      <c r="O59" t="n">
+        <v>69.01187863137507</v>
+      </c>
       <c r="P59" t="n">
-        <v>0</v>
+        <v>69.01187863137507</v>
       </c>
       <c r="Q59" t="n">
         <v>0.1777777777777778</v>
@@ -7521,6 +7892,15 @@
       </c>
       <c r="AQ59" t="n">
         <v>57</v>
+      </c>
+      <c r="AR59" t="n">
+        <v>28</v>
+      </c>
+      <c r="AS59" t="n">
+        <v>8612</v>
+      </c>
+      <c r="AT59" t="n">
+        <v>1068.994</v>
       </c>
     </row>
     <row r="60">
@@ -7570,8 +7950,14 @@
       <c r="M60" t="n">
         <v>23.17</v>
       </c>
+      <c r="N60" t="n">
+        <v>1169.093</v>
+      </c>
+      <c r="O60" t="n">
+        <v>50.45718601640052</v>
+      </c>
       <c r="P60" t="n">
-        <v>0</v>
+        <v>50.45718601640052</v>
       </c>
       <c r="Q60" t="n">
         <v>0.5225555555555556</v>
@@ -7637,6 +8023,15 @@
       </c>
       <c r="AQ60" t="n">
         <v>58</v>
+      </c>
+      <c r="AR60" t="n">
+        <v>27</v>
+      </c>
+      <c r="AS60" t="n">
+        <v>8609</v>
+      </c>
+      <c r="AT60" t="n">
+        <v>1169.093</v>
       </c>
     </row>
     <row r="61">
@@ -7678,8 +8073,14 @@
       <c r="M61" t="n">
         <v>27.64</v>
       </c>
+      <c r="N61" t="n">
+        <v>2399.245</v>
+      </c>
+      <c r="O61" t="n">
+        <v>86.80336468885672</v>
+      </c>
       <c r="P61" t="n">
-        <v>0</v>
+        <v>86.80336468885672</v>
       </c>
       <c r="Q61" t="n">
         <v>0.2197777777777778</v>
@@ -7745,6 +8146,15 @@
       </c>
       <c r="AQ61" t="n">
         <v>59</v>
+      </c>
+      <c r="AR61" t="n">
+        <v>35</v>
+      </c>
+      <c r="AS61" t="n">
+        <v>8789</v>
+      </c>
+      <c r="AT61" t="n">
+        <v>2399.245</v>
       </c>
     </row>
     <row r="62">
@@ -7786,8 +8196,14 @@
       <c r="M62" t="n">
         <v>14.58</v>
       </c>
+      <c r="N62" t="n">
+        <v>927.2140000000001</v>
+      </c>
+      <c r="O62" t="n">
+        <v>63.59492455418382</v>
+      </c>
       <c r="P62" t="n">
-        <v>0</v>
+        <v>63.59492455418382</v>
       </c>
       <c r="Q62" t="n">
         <v>0.2022222222222222</v>
@@ -7831,6 +8247,15 @@
       </c>
       <c r="AQ62" t="n">
         <v>60</v>
+      </c>
+      <c r="AR62" t="n">
+        <v>29</v>
+      </c>
+      <c r="AS62" t="n">
+        <v>8613</v>
+      </c>
+      <c r="AT62" t="n">
+        <v>927.2140000000001</v>
       </c>
     </row>
     <row r="63">
@@ -7887,7 +8312,7 @@
         <v>141.4883027522936</v>
       </c>
       <c r="P63" t="n">
-        <v>141.4883028</v>
+        <v>141.4883027522936</v>
       </c>
       <c r="Q63" t="n">
         <v>0.09777777777777778</v>
@@ -7982,7 +8407,7 @@
         <v>90.79391796322489</v>
       </c>
       <c r="P64" t="n">
-        <v>90.79391796</v>
+        <v>90.79391796322489</v>
       </c>
       <c r="Q64" t="n">
         <v>0.1844444444444444</v>
@@ -8104,7 +8529,7 @@
         <v>121.1313624678663</v>
       </c>
       <c r="P65" t="n">
-        <v>121.1313625</v>
+        <v>121.1313624678663</v>
       </c>
       <c r="Q65" t="n">
         <v>0.2028888888888889</v>
@@ -8221,7 +8646,7 @@
         <v>108.2682557487381</v>
       </c>
       <c r="P66" t="n">
-        <v>108.2682557</v>
+        <v>108.2682557487381</v>
       </c>
       <c r="Q66" t="n">
         <v>0.1366666666666667</v>
@@ -8338,7 +8763,7 @@
         <v>54.22249637155298</v>
       </c>
       <c r="P67" t="n">
-        <v>54.22249637</v>
+        <v>54.22249637155298</v>
       </c>
       <c r="Q67" t="n">
         <v>0.3177777777777778</v>
@@ -8450,7 +8875,7 @@
         <v>372.6573619631902</v>
       </c>
       <c r="P68" t="n">
-        <v>372.657362</v>
+        <v>372.6573619631902</v>
       </c>
       <c r="Q68" t="n">
         <v>0.1111111111111111</v>
@@ -8567,7 +8992,7 @@
         <v>28.3023493360572</v>
       </c>
       <c r="P69" t="n">
-        <v>28.30234934</v>
+        <v>28.3023493360572</v>
       </c>
       <c r="Q69" t="n">
         <v>0.2255555555555555</v>
@@ -8684,7 +9109,7 @@
         <v>91.31869158878504</v>
       </c>
       <c r="P70" t="n">
-        <v>91.31869159</v>
+        <v>91.31869158878504</v>
       </c>
       <c r="Q70" t="n">
         <v>0.1577777777777778</v>
@@ -8799,8 +9224,14 @@
       <c r="M71" t="n">
         <v>22.19</v>
       </c>
+      <c r="N71" t="n">
+        <v>1450.786</v>
+      </c>
+      <c r="O71" t="n">
+        <v>65.38017124831005</v>
+      </c>
       <c r="P71" t="n">
-        <v>0</v>
+        <v>65.38017124831005</v>
       </c>
       <c r="Q71" t="n">
         <v>0.2625555555555555</v>
@@ -8866,6 +9297,15 @@
       </c>
       <c r="AQ71" t="n">
         <v>69</v>
+      </c>
+      <c r="AR71" t="n">
+        <v>31</v>
+      </c>
+      <c r="AS71" t="n">
+        <v>8752</v>
+      </c>
+      <c r="AT71" t="n">
+        <v>1450.786</v>
       </c>
     </row>
     <row r="72">
@@ -8917,7 +9357,7 @@
         <v>147.8285923753666</v>
       </c>
       <c r="P72" t="n">
-        <v>147.8285924</v>
+        <v>147.8285923753666</v>
       </c>
       <c r="Q72" t="n">
         <v>0.1311111111111111</v>
@@ -9002,7 +9442,7 @@
         <v>642172</v>
       </c>
       <c r="P73" t="n">
-        <v>102912.1795</v>
+        <v>102912.1794871795</v>
       </c>
       <c r="Q73" t="n">
         <v>0.19</v>
@@ -9115,8 +9555,14 @@
       <c r="M74" t="n">
         <v>19.81</v>
       </c>
+      <c r="N74" t="n">
+        <v>1398.526</v>
+      </c>
+      <c r="O74" t="n">
+        <v>70.59697122665321</v>
+      </c>
       <c r="P74" t="n">
-        <v>0</v>
+        <v>70.59697122665321</v>
       </c>
       <c r="Q74" t="n">
         <v>0.25</v>
@@ -9182,6 +9628,15 @@
       </c>
       <c r="AQ74" t="n">
         <v>72</v>
+      </c>
+      <c r="AR74" t="n">
+        <v>25</v>
+      </c>
+      <c r="AS74" t="n">
+        <v>8920</v>
+      </c>
+      <c r="AT74" t="n">
+        <v>1398.526</v>
       </c>
     </row>
     <row r="75">
@@ -9228,8 +9683,14 @@
       <c r="M75" t="n">
         <v>22.12</v>
       </c>
+      <c r="N75" t="n">
+        <v>2176.827</v>
+      </c>
+      <c r="O75" t="n">
+        <v>98.40990054249548</v>
+      </c>
       <c r="P75" t="n">
-        <v>0</v>
+        <v>98.40990054249548</v>
       </c>
       <c r="Q75" t="n">
         <v>0.2072222222222223</v>
@@ -9295,6 +9756,15 @@
       </c>
       <c r="AQ75" t="n">
         <v>73</v>
+      </c>
+      <c r="AR75" t="n">
+        <v>24</v>
+      </c>
+      <c r="AS75" t="n">
+        <v>8913</v>
+      </c>
+      <c r="AT75" t="n">
+        <v>2176.827</v>
       </c>
     </row>
     <row r="76">
@@ -9345,8 +9815,14 @@
       <c r="M76" t="n">
         <v>4.16</v>
       </c>
+      <c r="N76" t="n">
+        <v>561.283</v>
+      </c>
+      <c r="O76" t="n">
+        <v>134.9237980769231</v>
+      </c>
       <c r="P76" t="n">
-        <v>0</v>
+        <v>134.9237980769231</v>
       </c>
       <c r="Q76" t="n">
         <v>0.2463333333333333</v>
@@ -9412,6 +9888,15 @@
       </c>
       <c r="AQ76" t="n">
         <v>74</v>
+      </c>
+      <c r="AR76" t="n">
+        <v>22</v>
+      </c>
+      <c r="AS76" t="n">
+        <v>8909</v>
+      </c>
+      <c r="AT76" t="n">
+        <v>804.037</v>
       </c>
     </row>
     <row r="77">
@@ -9461,8 +9946,14 @@
       <c r="M77" t="n">
         <v>15.49</v>
       </c>
+      <c r="N77" t="n">
+        <v>1530.148</v>
+      </c>
+      <c r="O77" t="n">
+        <v>98.78295674628792</v>
+      </c>
       <c r="P77" t="n">
-        <v>0</v>
+        <v>98.78295674628792</v>
       </c>
       <c r="Q77" t="n">
         <v>0.3631111111111112</v>
@@ -9528,6 +10019,15 @@
       </c>
       <c r="AQ77" t="n">
         <v>75</v>
+      </c>
+      <c r="AR77" t="n">
+        <v>21</v>
+      </c>
+      <c r="AS77" t="n">
+        <v>8904</v>
+      </c>
+      <c r="AT77" t="n">
+        <v>1530.148</v>
       </c>
     </row>
     <row r="78">
@@ -9577,8 +10077,14 @@
       <c r="M78" t="n">
         <v>4.66</v>
       </c>
+      <c r="N78" t="n">
+        <v>752.939</v>
+      </c>
+      <c r="O78" t="n">
+        <v>161.5748927038626</v>
+      </c>
       <c r="P78" t="n">
-        <v>0</v>
+        <v>161.5748927038626</v>
       </c>
       <c r="Q78" t="n">
         <v>0.2515555555555556</v>
@@ -9644,6 +10150,15 @@
       </c>
       <c r="AQ78" t="n">
         <v>76</v>
+      </c>
+      <c r="AR78" t="n">
+        <v>23</v>
+      </c>
+      <c r="AS78" t="n">
+        <v>8911</v>
+      </c>
+      <c r="AT78" t="n">
+        <v>752.939</v>
       </c>
     </row>
     <row r="79">
@@ -9685,8 +10200,14 @@
       <c r="M79" t="n">
         <v>10.51</v>
       </c>
+      <c r="N79" t="n">
+        <v>804.231</v>
+      </c>
+      <c r="O79" t="n">
+        <v>76.52055185537583</v>
+      </c>
       <c r="P79" t="n">
-        <v>0</v>
+        <v>76.52055185537583</v>
       </c>
       <c r="Q79" t="n">
         <v>0.3352222222222222</v>
@@ -9725,6 +10246,15 @@
       </c>
       <c r="AQ79" t="n">
         <v>77</v>
+      </c>
+      <c r="AR79" t="n">
+        <v>26</v>
+      </c>
+      <c r="AS79" t="n">
+        <v>8935</v>
+      </c>
+      <c r="AT79" t="n">
+        <v>804.231</v>
       </c>
     </row>
     <row r="80">

</xml_diff>